<commit_message>
Updated figs for publication
</commit_message>
<xml_diff>
--- a/Morphological_Analysis/TukeyHSD_M7_Transition.xlsx
+++ b/Morphological_Analysis/TukeyHSD_M7_Transition.xlsx
@@ -1,77 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28827"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/185965a385c69db2/Documents/Moquegua_Morphology/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_AB8D2DB2867279BE62A75152F32F6A71A944D31B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DB13E30-F438-4518-9BA5-B868E1966EB7}"/>
   <bookViews>
-    <workbookView xWindow="1440" yWindow="1440" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="TukeyHSD_M7_Transition" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="15">
-  <si>
-    <t>Trait</t>
-  </si>
-  <si>
-    <t>Comparison</t>
-  </si>
-  <si>
-    <t>diff</t>
-  </si>
-  <si>
-    <t>lwr</t>
-  </si>
-  <si>
-    <t>upr</t>
-  </si>
-  <si>
-    <t>p adj</t>
-  </si>
-  <si>
-    <t>Cupule_number</t>
-  </si>
-  <si>
-    <t>Transitional_Wari-Early_Huaracane</t>
-  </si>
-  <si>
-    <t>Transitional_Wari-Later_Tiwanaku</t>
-  </si>
-  <si>
-    <t>Diameter_mm</t>
-  </si>
-  <si>
-    <t>Length_mm</t>
-  </si>
-  <si>
-    <t>Mean_Cupule_Width(mm)</t>
-  </si>
-  <si>
-    <t>Mean_cupule_height(mm)</t>
-  </si>
-  <si>
-    <t>Mean_kernel_row</t>
-  </si>
-  <si>
-    <t>Total_Wt_g</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,25 +59,17 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -171,7 +107,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -205,7 +141,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -240,10 +175,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -416,311 +350,376 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
+    <row r="1" s="1" customFormat="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Trait</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Comparison</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>diff</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>lwr</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>upr</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p adj</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Cupule_number</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C2">
-        <v>-4.8174603174603092</v>
+        <v>-4.81746031746032</v>
       </c>
       <c r="D2">
-        <v>-6.7263344163030201</v>
+        <v>-6.726334416303024</v>
       </c>
       <c r="E2">
-        <v>-2.9085862186175979</v>
+        <v>-2.908586218617616</v>
       </c>
       <c r="F2">
-        <v>2.1243469872089801E-8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>8</v>
+        <v>2.12434698720898E-08</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Cupule_number</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C3">
-        <v>1.6956115779645189</v>
+        <v>1.695611577964508</v>
       </c>
       <c r="D3">
-        <v>0.2315719760345849</v>
+        <v>0.2315719760345791</v>
       </c>
       <c r="E3">
-        <v>3.1596511798944542</v>
+        <v>3.159651179894436</v>
       </c>
       <c r="F3">
-        <v>1.8437762865965879E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>0.01843776286596632</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Diameter_mm</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C4">
-        <v>0.90650793650794625</v>
+        <v>0.9065079365079178</v>
       </c>
       <c r="D4">
-        <v>-4.0149716362295864</v>
+        <v>-4.014971636229614</v>
       </c>
       <c r="E4">
-        <v>5.827987509245478</v>
+        <v>5.82798750924545</v>
       </c>
       <c r="F4">
-        <v>0.90159140686301376</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>8</v>
+        <v>0.9015914068630195</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Diameter_mm</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C5">
-        <v>3.8661484593837478</v>
+        <v>3.866148459383748</v>
       </c>
       <c r="D5">
-        <v>9.1545933766545851E-2</v>
+        <v>0.09154593376654585</v>
       </c>
       <c r="E5">
-        <v>7.6407509850009498</v>
+        <v>7.64075098500095</v>
       </c>
       <c r="F5">
-        <v>4.3285537240181908E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>7</v>
+        <v>0.04328553724018191</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Length_mm</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C6">
-        <v>1.745714285714328</v>
+        <v>1.745714285714051</v>
       </c>
       <c r="D6">
-        <v>-16.662071978277709</v>
+        <v>-16.66207197827799</v>
       </c>
       <c r="E6">
-        <v>20.153500549706369</v>
+        <v>20.15350054970609</v>
       </c>
       <c r="F6">
-        <v>0.97289817728729</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s">
-        <v>8</v>
+        <v>0.9728981772872985</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Length_mm</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C7">
-        <v>13.42084500466852</v>
+        <v>13.42084500466841</v>
       </c>
       <c r="D7">
-        <v>-0.69728258199890725</v>
+        <v>-0.6972825819990174</v>
       </c>
       <c r="E7">
-        <v>27.538972591335948</v>
+        <v>27.53897259133585</v>
       </c>
       <c r="F7">
-        <v>6.6402255317872472E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
+        <v>0.06640225531787536</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Mean_Cupule_Width(mm)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C8">
-        <v>2.014637960650794</v>
+        <v>2.014637960650801</v>
       </c>
       <c r="D8">
-        <v>0.88224236058406436</v>
+        <v>0.8822423605840712</v>
       </c>
       <c r="E8">
-        <v>3.147033560717523</v>
+        <v>3.147033560717531</v>
       </c>
       <c r="F8">
-        <v>1.064104650332354E-4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9" t="s">
-        <v>8</v>
+        <v>0.0001064104650332354</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Mean_Cupule_Width(mm)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C9">
-        <v>0.27866196192203502</v>
+        <v>0.2786619619220385</v>
       </c>
       <c r="D9">
-        <v>-0.58984581685395565</v>
+        <v>-0.5898458168539523</v>
       </c>
       <c r="E9">
-        <v>1.147169740698025</v>
+        <v>1.147169740698029</v>
       </c>
       <c r="F9">
-        <v>0.73060429830213303</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
+        <v>0.7306042983021274</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Mean_cupule_height(mm)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C10">
-        <v>0.95066356822222131</v>
+        <v>0.950663568222232</v>
       </c>
       <c r="D10">
-        <v>0.32918357727174641</v>
+        <v>0.329183577271757</v>
       </c>
       <c r="E10">
-        <v>1.572143559172696</v>
+        <v>1.572143559172707</v>
       </c>
       <c r="F10">
-        <v>1.0603360177745551E-3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>12</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
+        <v>0.001060336017774333</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mean_cupule_height(mm)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C11">
-        <v>0.31978452525817008</v>
+        <v>0.3197845252581715</v>
       </c>
       <c r="D11">
-        <v>-0.15686886907002481</v>
+        <v>-0.1568688690700235</v>
       </c>
       <c r="E11">
-        <v>0.79643791958636512</v>
+        <v>0.7964379195863664</v>
       </c>
       <c r="F11">
-        <v>0.25595834251625033</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" t="s">
-        <v>7</v>
+        <v>0.2559583425162474</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mean_kernel_row</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C12">
-        <v>-1.1111111121269741</v>
+        <v>-1.111111112127059</v>
       </c>
       <c r="D12">
-        <v>-6.2936372077527691</v>
+        <v>-6.293637207752854</v>
       </c>
       <c r="E12">
-        <v>4.0714149834988218</v>
+        <v>4.071414983498736</v>
       </c>
       <c r="F12">
-        <v>0.86908409569954048</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" t="s">
-        <v>8</v>
+        <v>0.8690840956995218</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mean_kernel_row</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C13">
-        <v>3.6884531592913148</v>
+        <v>3.68845315929128</v>
       </c>
       <c r="D13">
-        <v>-0.28636290984152879</v>
+        <v>-0.2863629098415643</v>
       </c>
       <c r="E13">
-        <v>7.6632692284241593</v>
+        <v>7.663269228424124</v>
       </c>
       <c r="F13">
-        <v>7.5292194335538243E-2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" t="s">
-        <v>7</v>
+        <v>0.07529219433554191</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Total_Wt_g</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Early_Huaracane</t>
+        </is>
       </c>
       <c r="C14">
-        <v>-0.50396825396823353</v>
+        <v>-0.5039682539682686</v>
       </c>
       <c r="D14">
-        <v>-2.1568803396443861</v>
+        <v>-2.156880339644419</v>
       </c>
       <c r="E14">
-        <v>1.1489438317079179</v>
+        <v>1.148943831707882</v>
       </c>
       <c r="F14">
-        <v>0.75314131387437466</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" t="s">
-        <v>8</v>
+        <v>0.7531413138743448</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Total_Wt_g</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Transitional_Wari-Later_Tiwanaku</t>
+        </is>
       </c>
       <c r="C15">
-        <v>0.63711017740430465</v>
+        <v>0.6371101774042853</v>
       </c>
       <c r="D15">
-        <v>-0.63061552195198889</v>
+        <v>-0.6306155219520078</v>
       </c>
       <c r="E15">
-        <v>1.904835876760598</v>
+        <v>1.904835876760578</v>
       </c>
       <c r="F15">
-        <v>0.46406674261244851</v>
+        <v>0.4640667426124698</v>
       </c>
     </row>
   </sheetData>

</xml_diff>